<commit_message>
[Doc]: bổ sung test report theo main tới #201 — 26 case API mới cho mic phòng ghi từng lượt, xoá lượt, tải bản ghi/bản gỡ băng, nghe lại câu nói, loại câu khỏi bản ghi, câu gửi muộn, giọng mẫu nghe lại và gắn tài liệu vào mục nghị sự; thay 3 case trỏ tới test đã đổi tên/bỏ (cách ghi âm giờ theo hình thức họp); cập nhật case UI ghi âm, lời nói, nội dung họp, ô chọn ngày giờ, Voice ID; thêm SYS-10; sinh lại 6 file Report 5.x (1129 test method)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/08-reports/test-reports/Report5.2.2_Integration_Test_API_Test.xlsx
+++ b/docs/08-reports/test-reports/Report5.2.2_Integration_Test_API_Test.xlsx
@@ -1323,7 +1323,7 @@
         <v>Issue Date</v>
       </c>
       <c r="F5" s="14" t="str">
-        <v>2026-10-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -1549,7 +1549,7 @@
     </row>
     <row r="12" ht="21.75" customHeight="1">
       <c r="A12" s="32" t="str">
-        <v>2026-10-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="B12" s="26" t="str">
         <v>1.1</v>
@@ -1561,7 +1561,7 @@
         <v>M</v>
       </c>
       <c r="E12" s="33" t="str">
-        <v>Regenerate: 1099 xUnit methods</v>
+        <v>Regenerate: 1129 xUnit methods</v>
       </c>
       <c r="F12" s="34" t="str"/>
       <c r="G12" s="31"/>
@@ -15256,7 +15256,7 @@
         <v>Number of TCs</v>
       </c>
       <c r="B4" s="110" t="n">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -15328,19 +15328,19 @@
         <v>Round 1</v>
       </c>
       <c r="B6" s="114" t="n">
-        <f>COUNTIF(F12:F62,"Passed")</f>
+        <f>COUNTIF(F12:F105,"Passed")</f>
         <v>0</v>
       </c>
       <c r="C6" s="114" t="n">
-        <f>COUNTIF(F12:F62,"Failed")</f>
+        <f>COUNTIF(F12:F105,"Failed")</f>
         <v>0</v>
       </c>
       <c r="D6" s="114" t="n">
         <f>B4-B6-C6-E6</f>
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="E6" s="114" t="n">
-        <f>COUNTIF(F12:F62,"Skipped")</f>
+        <f>COUNTIF(F12:F105,"Skipped")</f>
         <v>0</v>
       </c>
       <c r="F6" s="107"/>
@@ -15369,19 +15369,19 @@
         <v>Round 2</v>
       </c>
       <c r="B7" s="114" t="n">
-        <f>COUNTIF(I12:I62,"Passed")</f>
+        <f>COUNTIF(I12:I105,"Passed")</f>
         <v>0</v>
       </c>
       <c r="C7" s="114" t="n">
-        <f>COUNTIF(I12:I62,"Failed")</f>
+        <f>COUNTIF(I12:I105,"Failed")</f>
         <v>0</v>
       </c>
       <c r="D7" s="114" t="n">
         <f>B4-B7-C7-E7</f>
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="E7" s="114" t="n">
-        <f>COUNTIF(I12:I62,"Skipped")</f>
+        <f>COUNTIF(I12:I105,"Skipped")</f>
         <v>0</v>
       </c>
       <c r="F7" s="107"/>
@@ -15410,19 +15410,19 @@
         <v>Round 3</v>
       </c>
       <c r="B8" s="114" t="n">
-        <f>COUNTIF(L12:L62,"Passed")</f>
+        <f>COUNTIF(L12:L105,"Passed")</f>
         <v>0</v>
       </c>
       <c r="C8" s="114" t="n">
-        <f>COUNTIF(L12:L62,"Failed")</f>
+        <f>COUNTIF(L12:L105,"Failed")</f>
         <v>0</v>
       </c>
       <c r="D8" s="114" t="n">
         <f>B4-B8-C8-E8</f>
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="E8" s="114" t="n">
-        <f>COUNTIF(L12:L62,"Skipped")</f>
+        <f>COUNTIF(L12:L105,"Skipped")</f>
         <v>0</v>
       </c>
       <c r="F8" s="107"/>
@@ -15604,23 +15604,26 @@
       <c r="X12" s="112"/>
       <c r="Y12" s="112"/>
     </row>
-    <row r="13" ht="80.5" customHeight="1">
+    <row r="13" ht="167.5" customHeight="1">
       <c r="A13" s="120" t="str">
         <v>REC_API_IT02</v>
       </c>
       <c r="B13" s="120" t="str">
-        <v>Verify a browser capture is stored as such and codec parameters are accepted.</v>
+        <v>Verify the upload form carries only a file recorded elsewhere and codec parameters are accepted.</v>
       </c>
       <c r="C13" s="120" t="str">
-        <v>1. As the Secretary, POST a recording with file ghi-truc-tiep.webm of type audio/webm;codecs=opus, source=BrowserCapture and no durationMs.</v>
+        <v>1. As the Secretary, POST /api/meetings/&lt;id&gt;/recordings with consentConfirmed=true, a valid file and source=BrowserCapture.
+2. POST again with file ghi-ngoai.webm of type audio/webm;codecs=opus and no durationMs.
+3. GET /api/meetings/&lt;id&gt;/recordings.</v>
       </c>
       <c r="D13" s="120" t="str">
-        <v>1. HTTP 201 with code "MSG290".
-2. The item has source "BrowserCapture", contentType "audio/webm" and duration 0.</v>
+        <v>1. The form claiming a browser capture returns HTTP 400 with code "MSG291" ("Thông tin bản ghi không hợp lệ."): only the room mic records in the browser.
+2. The upload returns HTTP 201 with code "MSG290".
+3. The item has source "Upload", contentType "audio/webm", durationMs 0 and takes null.</v>
       </c>
       <c r="E13" s="120" t="str">
         <v>1. Backend is running.
-2. An InProgress meeting and its Secretary signed in.</v>
+2. An InProgress in-person meeting and its Secretary signed in.</v>
       </c>
       <c r="F13" s="121" t="str">
         <v>Pending</v>
@@ -16536,7 +16539,7 @@
       <c r="X37" s="112"/>
       <c r="Y37" s="112"/>
     </row>
-    <row r="38" ht="124.0" customHeight="1">
+    <row r="38" ht="153.0" customHeight="1">
       <c r="A38" s="120" t="str">
         <v>REC_API_IT17</v>
       </c>
@@ -16550,11 +16553,12 @@
       <c r="D38" s="120" t="str">
         <v>1. HTTP 200 with code "MSG318".
 2. clip.speakerId is the Member and clip.text is "Tôi đồng ý với dự thảo. Đề nghị biểu quyết.".
-3. The repeat returns the saved sentence without transcribing again.</v>
+3. The repeat returns the saved sentence without transcribing again.
+4. The sentence's audio is stored (audio/wav) and its line has hasAudio true; the list reports retentionDays 180.</v>
       </c>
       <c r="E38" s="120" t="str">
         <v>1. Backend is running.
-2. An InProgress meeting using per-microphone capture; the speech worker is running.</v>
+2. An InProgress Online or Hybrid meeting (captured per microphone); the speech worker is running.</v>
       </c>
       <c r="F38" s="121" t="str">
         <v>Pending</v>
@@ -16579,7 +16583,7 @@
       <c r="X38" s="112"/>
       <c r="Y38" s="112"/>
     </row>
-    <row r="39" ht="80.5" customHeight="1">
+    <row r="39" ht="95.0" customHeight="1">
       <c r="A39" s="120" t="str">
         <v>REC_API_IT18</v>
       </c>
@@ -16592,11 +16596,12 @@
       </c>
       <c r="D39" s="120" t="str">
         <v>1. HTTP 204 No Content.
-2. The list is empty.</v>
+2. The list is empty.
+3. No audio file is stored.</v>
       </c>
       <c r="E39" s="120" t="str">
         <v>1. Backend is running.
-2. An InProgress per-microphone meeting; the speech worker is running.</v>
+2. An InProgress Online or Hybrid meeting (captured per microphone); the speech worker is running.</v>
       </c>
       <c r="F39" s="121" t="str">
         <v>Pending</v>
@@ -16621,21 +16626,23 @@
       <c r="X39" s="112"/>
       <c r="Y39" s="112"/>
     </row>
-    <row r="40" ht="138.5" customHeight="1">
+    <row r="40" ht="211.0" customHeight="1">
       <c r="A40" s="120" t="str">
         <v>REC_API_IT19</v>
       </c>
       <c r="B40" s="120" t="str">
-        <v>Verify sentences are accepted only from people of a running per-microphone meeting.</v>
+        <v>Verify sentences are accepted only from people of a running meeting joined from afar.</v>
       </c>
       <c r="C40" s="120" t="str">
-        <v>1. As the Member, send a clip to a meeting using whole-room capture.
-2. Send a clip to a Published meeting that has not started.
-3. As an outsider, send a clip to a running per-microphone meeting.</v>
+        <v>1. As the Member, send a sentence to an InProgress in-person meeting (recorded by the room mic) and GET its speech-clips.
+2. Send a sentence to a Published meeting that has not started.
+3. As an outsider, send a sentence to a running Online meeting.
+4. As the organizer, who is not on the roster, GET /api/meetings/&lt;id&gt;/speech-clips.</v>
       </c>
       <c r="D40" s="120" t="str">
-        <v>1. Room capture and not started: HTTP 409 with code "MSG320"; canCapture is false.
-2. Outsider: HTTP 404.</v>
+        <v>1. In-person and not started: HTTP 409 with code "MSG320" ("Cuộc họp trực tiếp không ghi theo micro từng người, hoặc cuộc họp không còn đang diễn ra."); canCapture is false for the in-person meeting.
+2. Outsider: HTTP 404.
+3. Organizer: HTTP 404; no one's words are theirs to read.</v>
       </c>
       <c r="E40" s="120" t="str">
         <v>1. Backend is running.
@@ -16680,7 +16687,7 @@
       </c>
       <c r="E41" s="120" t="str">
         <v>1. Backend is running.
-2. An InProgress per-microphone meeting.</v>
+2. An InProgress Online or Hybrid meeting (captured per microphone).</v>
       </c>
       <c r="F41" s="121" t="str">
         <v>Pending</v>
@@ -16722,7 +16729,7 @@
       </c>
       <c r="E42" s="120" t="str">
         <v>1. Backend is running.
-2. An InProgress per-microphone meeting.</v>
+2. An InProgress Online or Hybrid meeting (captured per microphone).</v>
       </c>
       <c r="F42" s="121" t="str">
         <v>Pending</v>
@@ -16893,7 +16900,7 @@
     </row>
     <row r="47" ht="24" customHeight="1">
       <c r="A47" s="120" t="str">
-        <v>PUT /api/meetings/{id}/capture-mode</v>
+        <v>PUT /api/meetings/{id}/speech-clips/{clientId}</v>
       </c>
       <c r="B47" s="120"/>
       <c r="C47" s="120"/>
@@ -16920,26 +16927,26 @@
       <c r="X47" s="112"/>
       <c r="Y47" s="112"/>
     </row>
-    <row r="48" ht="138.5" customHeight="1">
+    <row r="48" ht="124.0" customHeight="1">
       <c r="A48" s="120" t="str">
         <v>REC_API_IT24</v>
       </c>
       <c r="B48" s="120" t="str">
-        <v>Verify the Chair or a Secretary picks the capture mode until the meeting starts.</v>
+        <v>Verify a meeting joined from afar is captured per microphone (Online, Hybrid).</v>
       </c>
       <c r="C48" s="120" t="str">
-        <v>1. As the Secretary of a Published meeting, GET the clip list and PUT /api/meetings/&lt;id&gt;/capture-mode with { "mode": "Room" }.
-2. As the Member, try to change the mode.
-3. Start the meeting and try again as the Secretary.</v>
+        <v>1. As the Member of an InProgress Online meeting, GET /api/meetings/&lt;id&gt;/speech-clips.
+2. Send a sentence with PUT /api/meetings/&lt;id&gt;/speech-clips/&lt;new UUID&gt;.
+3. Repeat for a Hybrid meeting.</v>
       </c>
       <c r="D48" s="120" t="str">
-        <v>1. canChangeMode is true; the change returns HTTP 200 with code "MSG324" ("Đã đổi cách ghi âm.") and captureMode "Room".
-2. The Member is refused.
-3. After the meeting starts the change is refused.</v>
+        <v>1. canCapture is true.
+2. The sentence returns HTTP 200 with code "MSG318" ("Đã ghi câu nói.").
+3. The capture mode follows the meeting's Hình thức; there is no capture-mode setting to change.</v>
       </c>
       <c r="E48" s="120" t="str">
         <v>1. Backend is running.
-2. A Published meeting with Chair, Secretary and Member.</v>
+2. InProgress Online and Hybrid meetings with the Member on their roster; the speech worker is running.</v>
       </c>
       <c r="F48" s="121" t="str">
         <v>Pending</v>
@@ -17471,8 +17478,1641 @@
       <c r="X62" s="112"/>
       <c r="Y62" s="112"/>
     </row>
+    <row r="63" ht="24" customHeight="1">
+      <c r="A63" s="120" t="str">
+        <v>POST /api/meetings/{id}/recordings</v>
+      </c>
+      <c r="B63" s="120"/>
+      <c r="C63" s="120"/>
+      <c r="D63" s="120"/>
+      <c r="E63" s="120"/>
+      <c r="F63" s="121"/>
+      <c r="G63" s="122"/>
+      <c r="H63" s="121"/>
+      <c r="I63" s="121"/>
+      <c r="J63" s="122"/>
+      <c r="K63" s="121"/>
+      <c r="L63" s="121"/>
+      <c r="M63" s="123"/>
+      <c r="N63" s="121"/>
+      <c r="O63" s="124"/>
+      <c r="P63" s="125"/>
+      <c r="Q63" s="112"/>
+      <c r="R63" s="112"/>
+      <c r="S63" s="112"/>
+      <c r="T63" s="112"/>
+      <c r="U63" s="112"/>
+      <c r="V63" s="112"/>
+      <c r="W63" s="112"/>
+      <c r="X63" s="112"/>
+      <c r="Y63" s="112"/>
+    </row>
+    <row r="64" ht="124.0" customHeight="1">
+      <c r="A64" s="120" t="str">
+        <v>REC_API_IT32</v>
+      </c>
+      <c r="B64" s="120" t="str">
+        <v>Verify an online meeting has no room recording (InProgress, Ended).</v>
+      </c>
+      <c r="C64" s="120" t="str">
+        <v>1. As the Secretary of an Online meeting, POST /api/meetings/&lt;id&gt;/recordings with a valid form.
+2. GET /api/meetings/&lt;id&gt;/recordings.
+3. Repeat for an in-person meeting in the same status.</v>
+      </c>
+      <c r="D64" s="120" t="str">
+        <v>1. Online: HTTP 409 with code "MSG358" ("Cuộc họp trực tuyến ghi theo micro từng người, không có bản ghi phòng."); canUpload is false and no file is stored.
+2. In-person: the upload returns HTTP 201 with code "MSG290".</v>
+      </c>
+      <c r="E64" s="120" t="str">
+        <v>1. Backend is running.
+2. InProgress and Ended meetings, Online and in-person, each with its Secretary.
+3. File storage is configured.</v>
+      </c>
+      <c r="F64" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G64" s="122" t="str"/>
+      <c r="H64" s="121" t="str"/>
+      <c r="I64" s="121" t="str"/>
+      <c r="J64" s="122" t="str"/>
+      <c r="K64" s="121" t="str"/>
+      <c r="L64" s="121" t="str"/>
+      <c r="M64" s="123" t="str"/>
+      <c r="N64" s="121" t="str"/>
+      <c r="O64" s="124" t="str"/>
+      <c r="P64" s="125"/>
+      <c r="Q64" s="112"/>
+      <c r="R64" s="112"/>
+      <c r="S64" s="112"/>
+      <c r="T64" s="112"/>
+      <c r="U64" s="112"/>
+      <c r="V64" s="112"/>
+      <c r="W64" s="112"/>
+      <c r="X64" s="112"/>
+      <c r="Y64" s="112"/>
+    </row>
+    <row r="65" ht="24" customHeight="1">
+      <c r="A65" s="120" t="str">
+        <v>POST /api/meetings/{id}/recordings/takes</v>
+      </c>
+      <c r="B65" s="120"/>
+      <c r="C65" s="120"/>
+      <c r="D65" s="120"/>
+      <c r="E65" s="120"/>
+      <c r="F65" s="121"/>
+      <c r="G65" s="122"/>
+      <c r="H65" s="121"/>
+      <c r="I65" s="121"/>
+      <c r="J65" s="122"/>
+      <c r="K65" s="121"/>
+      <c r="L65" s="121"/>
+      <c r="M65" s="123"/>
+      <c r="N65" s="121"/>
+      <c r="O65" s="124"/>
+      <c r="P65" s="125"/>
+      <c r="Q65" s="112"/>
+      <c r="R65" s="112"/>
+      <c r="S65" s="112"/>
+      <c r="T65" s="112"/>
+      <c r="U65" s="112"/>
+      <c r="V65" s="112"/>
+      <c r="W65" s="112"/>
+      <c r="X65" s="112"/>
+      <c r="Y65" s="112"/>
+    </row>
+    <row r="66" ht="370.5" customHeight="1">
+      <c r="A66" s="120" t="str">
+        <v>REC_API_IT33</v>
+      </c>
+      <c r="B66" s="120" t="str">
+        <v>Verify the first take streams in parts and becomes the meeting's room recording.</v>
+      </c>
+      <c r="C66" s="120" t="str">
+        <v>1. As the Member and the Secretary, GET /api/meetings/&lt;id&gt;/recordings and read canRecord.
+2. As the Secretary, POST /api/meetings/&lt;id&gt;/recordings/takes with body { "consentConfirmed": true, "consentPurpose": "Lập biên bản phiên họp" }.
+3. As the Member, GET the list and GET /api/recordings/&lt;take&gt;/playback.
+4. As the Secretary, PUT /api/recordings/&lt;take&gt;/parts/1 with the first full part, send part 1 again, then PUT /api/recordings/&lt;take&gt;/parts/2?final=true with the shorter last part. Each part is application/octet-stream of exactly partSize bytes; part 1 starts with a WAV header for 16 kHz mono 16-bit PCM.
+… (continued in the test source)</v>
+      </c>
+      <c r="D66" s="120" t="str">
+        <v>1. canRecord is true for the Secretary and false for the Member.
+2. The take returns HTTP 201 with recordingId and partSize.
+3. While recording, everyone sees one item with status "Pending", created by the Secretary; only the Secretary may close it; playback returns HTTP 404.
+4. Each part, including the repeated part 1, returns HTTP 204.
+5. Both completions return HTTP 200 with code "MSG363" ("Đã lưu lượt ghi."), the same recordingId and appended false.
+6. The item is "Available", source "BrowserCapture", transcriptStatus "Pending", with the purpose, the duration of the PCM and one take at offset 0; the stored WAV header carries the final length.
+7. The audit log records the take started and saved by the Secretary.</v>
+      </c>
+      <c r="E66" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress in-person meeting with Secretary and Member.
+3. File storage is configured.</v>
+      </c>
+      <c r="F66" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G66" s="122" t="str"/>
+      <c r="H66" s="121" t="str"/>
+      <c r="I66" s="121" t="str"/>
+      <c r="J66" s="122" t="str"/>
+      <c r="K66" s="121" t="str"/>
+      <c r="L66" s="121" t="str"/>
+      <c r="M66" s="123" t="str"/>
+      <c r="N66" s="121" t="str"/>
+      <c r="O66" s="124" t="str"/>
+      <c r="P66" s="125"/>
+      <c r="Q66" s="112"/>
+      <c r="R66" s="112"/>
+      <c r="S66" s="112"/>
+      <c r="T66" s="112"/>
+      <c r="U66" s="112"/>
+      <c r="V66" s="112"/>
+      <c r="W66" s="112"/>
+      <c r="X66" s="112"/>
+      <c r="Y66" s="112"/>
+    </row>
+    <row r="67" ht="225.5" customHeight="1">
+      <c r="A67" s="120" t="str">
+        <v>REC_API_IT34</v>
+      </c>
+      <c r="B67" s="120" t="str">
+        <v>Verify a later take is appended to the room recording and the whole is transcribed again.</v>
+      </c>
+      <c r="C67" s="120" t="str">
+        <v>1. As the Secretary, record and complete a first take; let the speech worker finish.
+2. Ten minutes later, POST /api/meetings/&lt;id&gt;/recordings/takes with consentConfirmed=false, stream a second take and complete it.
+3. GET the list, then let the worker run and GET /api/recordings/&lt;room&gt;/transcript.</v>
+      </c>
+      <c r="D67" s="120" t="str">
+        <v>1. The second take needs no new consent; completing returns code "MSG363" with the room recording's id and appended true.
+2. There is still one item; it lists two takes, the second at the end of the first, with its own duration and start time; transcriptStatus is "Pending".
+3. The stored file is the first take followed by the second without its header; the whole file is transcribed and the transcript ends "Completed".
+4. No separate recording is left for the second take.</v>
+      </c>
+      <c r="E67" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress in-person meeting; signed in as its Secretary; speech worker running.</v>
+      </c>
+      <c r="F67" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G67" s="122" t="str"/>
+      <c r="H67" s="121" t="str"/>
+      <c r="I67" s="121" t="str"/>
+      <c r="J67" s="122" t="str"/>
+      <c r="K67" s="121" t="str"/>
+      <c r="L67" s="121" t="str"/>
+      <c r="M67" s="123" t="str"/>
+      <c r="N67" s="121" t="str"/>
+      <c r="O67" s="124" t="str"/>
+      <c r="P67" s="125"/>
+      <c r="Q67" s="112"/>
+      <c r="R67" s="112"/>
+      <c r="S67" s="112"/>
+      <c r="T67" s="112"/>
+      <c r="U67" s="112"/>
+      <c r="V67" s="112"/>
+      <c r="W67" s="112"/>
+      <c r="X67" s="112"/>
+      <c r="Y67" s="112"/>
+    </row>
+    <row r="68" ht="24" customHeight="1">
+      <c r="A68" s="120" t="str">
+        <v>POST /api/recordings/{id}/complete</v>
+      </c>
+      <c r="B68" s="120"/>
+      <c r="C68" s="120"/>
+      <c r="D68" s="120"/>
+      <c r="E68" s="120"/>
+      <c r="F68" s="121"/>
+      <c r="G68" s="122"/>
+      <c r="H68" s="121"/>
+      <c r="I68" s="121"/>
+      <c r="J68" s="122"/>
+      <c r="K68" s="121"/>
+      <c r="L68" s="121"/>
+      <c r="M68" s="123"/>
+      <c r="N68" s="121"/>
+      <c r="O68" s="124"/>
+      <c r="P68" s="125"/>
+      <c r="Q68" s="112"/>
+      <c r="R68" s="112"/>
+      <c r="S68" s="112"/>
+      <c r="T68" s="112"/>
+      <c r="U68" s="112"/>
+      <c r="V68" s="112"/>
+      <c r="W68" s="112"/>
+      <c r="X68" s="112"/>
+      <c r="Y68" s="112"/>
+    </row>
+    <row r="69" ht="124.0" customHeight="1">
+      <c r="A69" s="120" t="str">
+        <v>REC_API_IT35</v>
+      </c>
+      <c r="B69" s="120" t="str">
+        <v>Verify a take appended while the room recording is being transcribed makes that run start over.</v>
+      </c>
+      <c r="C69" s="120" t="str">
+        <v>1. As the Secretary, record and complete a take.
+2. While the speech worker transcribes it, record and complete a second take.
+3. GET /api/recordings/&lt;room&gt;/transcript, then let the worker run again.</v>
+      </c>
+      <c r="D69" s="120" t="str">
+        <v>1. The result of the shorter file is discarded: the transcript is "Pending" with no segments.
+2. The next run transcribes the whole room recording.</v>
+      </c>
+      <c r="E69" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress in-person meeting; signed in as its Secretary; speech worker running.</v>
+      </c>
+      <c r="F69" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G69" s="122" t="str"/>
+      <c r="H69" s="121" t="str"/>
+      <c r="I69" s="121" t="str"/>
+      <c r="J69" s="122" t="str"/>
+      <c r="K69" s="121" t="str"/>
+      <c r="L69" s="121" t="str"/>
+      <c r="M69" s="123" t="str"/>
+      <c r="N69" s="121" t="str"/>
+      <c r="O69" s="124" t="str"/>
+      <c r="P69" s="125"/>
+      <c r="Q69" s="112"/>
+      <c r="R69" s="112"/>
+      <c r="S69" s="112"/>
+      <c r="T69" s="112"/>
+      <c r="U69" s="112"/>
+      <c r="V69" s="112"/>
+      <c r="W69" s="112"/>
+      <c r="X69" s="112"/>
+      <c r="Y69" s="112"/>
+    </row>
+    <row r="70" ht="24" customHeight="1">
+      <c r="A70" s="120" t="str">
+        <v>POST /api/meetings/{id}/recordings/takes</v>
+      </c>
+      <c r="B70" s="120"/>
+      <c r="C70" s="120"/>
+      <c r="D70" s="120"/>
+      <c r="E70" s="120"/>
+      <c r="F70" s="121"/>
+      <c r="G70" s="122"/>
+      <c r="H70" s="121"/>
+      <c r="I70" s="121"/>
+      <c r="J70" s="122"/>
+      <c r="K70" s="121"/>
+      <c r="L70" s="121"/>
+      <c r="M70" s="123"/>
+      <c r="N70" s="121"/>
+      <c r="O70" s="124"/>
+      <c r="P70" s="125"/>
+      <c r="Q70" s="112"/>
+      <c r="R70" s="112"/>
+      <c r="S70" s="112"/>
+      <c r="T70" s="112"/>
+      <c r="U70" s="112"/>
+      <c r="V70" s="112"/>
+      <c r="W70" s="112"/>
+      <c r="X70" s="112"/>
+      <c r="Y70" s="112"/>
+    </row>
+    <row r="71" ht="240.0" customHeight="1">
+      <c r="A71" s="120" t="str">
+        <v>REC_API_IT36</v>
+      </c>
+      <c r="B71" s="120" t="str">
+        <v>Verify the room mic switches on only for the Secretary of a running in-person meeting.</v>
+      </c>
+      <c r="C71" s="120" t="str">
+        <v>1. As the Member, then as an outsider, POST /api/meetings/&lt;id&gt;/recordings/takes.
+2. As the Secretary, POST with consentConfirmed=false for the first take.
+3. As the Secretary of an Online meeting, and of an Ended in-person meeting, POST a take.
+4. As the Secretary, open a take, then POST another one.
+5. DELETE /api/recordings/&lt;open take&gt;.</v>
+      </c>
+      <c r="D71" s="120" t="str">
+        <v>1. Member: HTTP 403 with code "MSG295" ("Chỉ Thư ký cuộc họp được quản lý bản ghi."). Outsider: HTTP 404.
+2. No consent before the first take: HTTP 400 with code "MSG291" and an error on consentConfirmed.
+3. Online: HTTP 409 "MSG358". Ended: HTTP 409 "MSG359" ("Chỉ bật mic phòng khi cuộc họp đang diễn ra.").
+4. A second open take: HTTP 409 "MSG360" ("Mic phòng đang ghi ở một máy khác.").
+5. Deleting the open take: HTTP 409 "MSG364" ("Mic phòng đang ghi lượt này. Tắt mic để lưu rồi mới xoá được."); the file stays.</v>
+      </c>
+      <c r="E71" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress in-person meeting with Secretary, Member and an outsider; an Online and an Ended meeting.</v>
+      </c>
+      <c r="F71" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G71" s="122" t="str"/>
+      <c r="H71" s="121" t="str"/>
+      <c r="I71" s="121" t="str"/>
+      <c r="J71" s="122" t="str"/>
+      <c r="K71" s="121" t="str"/>
+      <c r="L71" s="121" t="str"/>
+      <c r="M71" s="123" t="str"/>
+      <c r="N71" s="121" t="str"/>
+      <c r="O71" s="124" t="str"/>
+      <c r="P71" s="125"/>
+      <c r="Q71" s="112"/>
+      <c r="R71" s="112"/>
+      <c r="S71" s="112"/>
+      <c r="T71" s="112"/>
+      <c r="U71" s="112"/>
+      <c r="V71" s="112"/>
+      <c r="W71" s="112"/>
+      <c r="X71" s="112"/>
+      <c r="Y71" s="112"/>
+    </row>
+    <row r="72" ht="24" customHeight="1">
+      <c r="A72" s="120" t="str">
+        <v>PUT /api/recordings/{id}/parts/{n}</v>
+      </c>
+      <c r="B72" s="120"/>
+      <c r="C72" s="120"/>
+      <c r="D72" s="120"/>
+      <c r="E72" s="120"/>
+      <c r="F72" s="121"/>
+      <c r="G72" s="122"/>
+      <c r="H72" s="121"/>
+      <c r="I72" s="121"/>
+      <c r="J72" s="122"/>
+      <c r="K72" s="121"/>
+      <c r="L72" s="121"/>
+      <c r="M72" s="123"/>
+      <c r="N72" s="121"/>
+      <c r="O72" s="124"/>
+      <c r="P72" s="125"/>
+      <c r="Q72" s="112"/>
+      <c r="R72" s="112"/>
+      <c r="S72" s="112"/>
+      <c r="T72" s="112"/>
+      <c r="U72" s="112"/>
+      <c r="V72" s="112"/>
+      <c r="W72" s="112"/>
+      <c r="X72" s="112"/>
+      <c r="Y72" s="112"/>
+    </row>
+    <row r="73" ht="225.5" customHeight="1">
+      <c r="A73" s="120" t="str">
+        <v>REC_API_IT37</v>
+      </c>
+      <c r="B73" s="120" t="str">
+        <v>Verify parts come in order, at their size, from the take's maker, until it is saved.</v>
+      </c>
+      <c r="C73" s="120" t="str">
+        <v>1. As the Secretary, open a take.
+2. PUT part 1 as plain noise with no WAV header; as a WAV at 44.1 kHz; two bytes short of partSize; PUT part 0; PUT part 2 before part 1.
+3. As the Chair, PUT part 1 and POST /api/recordings/&lt;take&gt;/complete.
+4. As the Secretary, PUT part 1, PUT part 2?final=true with 10 bytes, then PUT part 3.
+5. Complete the take, then PUT part 2 again.</v>
+      </c>
+      <c r="D73" s="120" t="str">
+        <v>1. Every malformed or out-of-order part returns HTTP 400 with code "MSG361" ("Phần âm thanh gửi lên không hợp lệ.").
+2. Chair: the part returns HTTP 404; completing returns HTTP 403 "MSG295".
+3. Valid parts return HTTP 204; a part after the short last part returns HTTP 400 "MSG361".
+4. After the take is saved, a part returns HTTP 409 "MSG362" ("Lượt ghi này đã được lưu, không thêm tiếng vào được nữa.").</v>
+      </c>
+      <c r="E73" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress in-person meeting with its Secretary and Chair.</v>
+      </c>
+      <c r="F73" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G73" s="122" t="str"/>
+      <c r="H73" s="121" t="str"/>
+      <c r="I73" s="121" t="str"/>
+      <c r="J73" s="122" t="str"/>
+      <c r="K73" s="121" t="str"/>
+      <c r="L73" s="121" t="str"/>
+      <c r="M73" s="123" t="str"/>
+      <c r="N73" s="121" t="str"/>
+      <c r="O73" s="124" t="str"/>
+      <c r="P73" s="125"/>
+      <c r="Q73" s="112"/>
+      <c r="R73" s="112"/>
+      <c r="S73" s="112"/>
+      <c r="T73" s="112"/>
+      <c r="U73" s="112"/>
+      <c r="V73" s="112"/>
+      <c r="W73" s="112"/>
+      <c r="X73" s="112"/>
+      <c r="Y73" s="112"/>
+    </row>
+    <row r="74" ht="95.0" customHeight="1">
+      <c r="A74" s="120" t="str">
+        <v>REC_API_IT38</v>
+      </c>
+      <c r="B74" s="120" t="str">
+        <v>Verify a take cannot grow past the recording limit.</v>
+      </c>
+      <c r="C74" s="120" t="str">
+        <v>1. As the Secretary, open a take.
+2. PUT parts one after another until their total reaches Recordings:MaxUploadMegabytes.
+3. PUT one more part.</v>
+      </c>
+      <c r="D74" s="120" t="str">
+        <v>1. Parts within the limit return HTTP 204.
+2. The part past the limit returns HTTP 413 with code "MSG293" ("Bản ghi vượt quá 300 MB." with the configured size).</v>
+      </c>
+      <c r="E74" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress in-person meeting; a small Recordings:MaxUploadMegabytes on the test server.</v>
+      </c>
+      <c r="F74" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G74" s="122" t="str"/>
+      <c r="H74" s="121" t="str"/>
+      <c r="I74" s="121" t="str"/>
+      <c r="J74" s="122" t="str"/>
+      <c r="K74" s="121" t="str"/>
+      <c r="L74" s="121" t="str"/>
+      <c r="M74" s="123" t="str"/>
+      <c r="N74" s="121" t="str"/>
+      <c r="O74" s="124" t="str"/>
+      <c r="P74" s="125"/>
+      <c r="Q74" s="112"/>
+      <c r="R74" s="112"/>
+      <c r="S74" s="112"/>
+      <c r="T74" s="112"/>
+      <c r="U74" s="112"/>
+      <c r="V74" s="112"/>
+      <c r="W74" s="112"/>
+      <c r="X74" s="112"/>
+      <c r="Y74" s="112"/>
+    </row>
+    <row r="75" ht="24" customHeight="1">
+      <c r="A75" s="120" t="str">
+        <v>POST /api/recordings/{id}/complete</v>
+      </c>
+      <c r="B75" s="120"/>
+      <c r="C75" s="120"/>
+      <c r="D75" s="120"/>
+      <c r="E75" s="120"/>
+      <c r="F75" s="121"/>
+      <c r="G75" s="122"/>
+      <c r="H75" s="121"/>
+      <c r="I75" s="121"/>
+      <c r="J75" s="122"/>
+      <c r="K75" s="121"/>
+      <c r="L75" s="121"/>
+      <c r="M75" s="123"/>
+      <c r="N75" s="121"/>
+      <c r="O75" s="124"/>
+      <c r="P75" s="125"/>
+      <c r="Q75" s="112"/>
+      <c r="R75" s="112"/>
+      <c r="S75" s="112"/>
+      <c r="T75" s="112"/>
+      <c r="U75" s="112"/>
+      <c r="V75" s="112"/>
+      <c r="W75" s="112"/>
+      <c r="X75" s="112"/>
+      <c r="Y75" s="112"/>
+    </row>
+    <row r="76" ht="124.0" customHeight="1">
+      <c r="A76" s="120" t="str">
+        <v>REC_API_IT39</v>
+      </c>
+      <c r="B76" s="120" t="str">
+        <v>Verify a take the mic heard nothing in is dropped.</v>
+      </c>
+      <c r="C76" s="120" t="str">
+        <v>1. As the Secretary, open a take and complete it without sending any part.
+2. GET the list.
+3. Open a new take.</v>
+      </c>
+      <c r="D76" s="120" t="str">
+        <v>1. HTTP 200 with code "MSG365" ("Mic chưa thu được tiếng nào nên lượt này không được lưu.") and recordingId null.
+2. The list is empty and no file is stored.
+3. The mic switches on again normally (HTTP 201).</v>
+      </c>
+      <c r="E76" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress in-person meeting; signed in as its Secretary.</v>
+      </c>
+      <c r="F76" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G76" s="122" t="str"/>
+      <c r="H76" s="121" t="str"/>
+      <c r="I76" s="121" t="str"/>
+      <c r="J76" s="122" t="str"/>
+      <c r="K76" s="121" t="str"/>
+      <c r="L76" s="121" t="str"/>
+      <c r="M76" s="123" t="str"/>
+      <c r="N76" s="121" t="str"/>
+      <c r="O76" s="124" t="str"/>
+      <c r="P76" s="125"/>
+      <c r="Q76" s="112"/>
+      <c r="R76" s="112"/>
+      <c r="S76" s="112"/>
+      <c r="T76" s="112"/>
+      <c r="U76" s="112"/>
+      <c r="V76" s="112"/>
+      <c r="W76" s="112"/>
+      <c r="X76" s="112"/>
+      <c r="Y76" s="112"/>
+    </row>
+    <row r="77" ht="109.5" customHeight="1">
+      <c r="A77" s="120" t="str">
+        <v>REC_API_IT40</v>
+      </c>
+      <c r="B77" s="120" t="str">
+        <v>Verify a take left open is saved by the server once no part has come for hours.</v>
+      </c>
+      <c r="C77" s="120" t="str">
+        <v>1. As the Secretary, open a take and send part 1, then close the browser.
+2. Run the idle-take sweep at once, and again after 13 hours without parts.
+3. GET the list.</v>
+      </c>
+      <c r="D77" s="120" t="str">
+        <v>1. The first sweep saves nothing.
+2. After 13 hours the take is saved: the item is "Available".
+3. The audit log records the take saved with no actor (the server).</v>
+      </c>
+      <c r="E77" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress in-person meeting; the server clock can be advanced.</v>
+      </c>
+      <c r="F77" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G77" s="122" t="str"/>
+      <c r="H77" s="121" t="str"/>
+      <c r="I77" s="121" t="str"/>
+      <c r="J77" s="122" t="str"/>
+      <c r="K77" s="121" t="str"/>
+      <c r="L77" s="121" t="str"/>
+      <c r="M77" s="123" t="str"/>
+      <c r="N77" s="121" t="str"/>
+      <c r="O77" s="124" t="str"/>
+      <c r="P77" s="125"/>
+      <c r="Q77" s="112"/>
+      <c r="R77" s="112"/>
+      <c r="S77" s="112"/>
+      <c r="T77" s="112"/>
+      <c r="U77" s="112"/>
+      <c r="V77" s="112"/>
+      <c r="W77" s="112"/>
+      <c r="X77" s="112"/>
+      <c r="Y77" s="112"/>
+    </row>
+    <row r="78" ht="24" customHeight="1">
+      <c r="A78" s="120" t="str">
+        <v>DELETE /api/recordings/{id}/takes/{take}</v>
+      </c>
+      <c r="B78" s="120"/>
+      <c r="C78" s="120"/>
+      <c r="D78" s="120"/>
+      <c r="E78" s="120"/>
+      <c r="F78" s="121"/>
+      <c r="G78" s="122"/>
+      <c r="H78" s="121"/>
+      <c r="I78" s="121"/>
+      <c r="J78" s="122"/>
+      <c r="K78" s="121"/>
+      <c r="L78" s="121"/>
+      <c r="M78" s="123"/>
+      <c r="N78" s="121"/>
+      <c r="O78" s="124"/>
+      <c r="P78" s="125"/>
+      <c r="Q78" s="112"/>
+      <c r="R78" s="112"/>
+      <c r="S78" s="112"/>
+      <c r="T78" s="112"/>
+      <c r="U78" s="112"/>
+      <c r="V78" s="112"/>
+      <c r="W78" s="112"/>
+      <c r="X78" s="112"/>
+      <c r="Y78" s="112"/>
+    </row>
+    <row r="79" ht="240.0" customHeight="1">
+      <c r="A79" s="120" t="str">
+        <v>REC_API_IT41</v>
+      </c>
+      <c r="B79" s="120" t="str">
+        <v>Verify a take is cut out of the room recording and its lines out of the transcript, keeping the rest.</v>
+      </c>
+      <c r="C79" s="120" t="str">
+        <v>1. As the Secretary, record three takes and let the transcript finish with one line in each take.
+2. Correct the third line and name SPEAKER_00 as the Chair.
+3. As the Member, DELETE /api/recordings/&lt;room&gt;/takes/2. As the Secretary, DELETE take 4, then take 2.
+4. GET the list and the transcript.
+5. DELETE take 2 again, then take 1.</v>
+      </c>
+      <c r="D79" s="120" t="str">
+        <v>1. Member: HTTP 403 "MSG295". Take 4: HTTP 404.
+2. Deleting take 2: HTTP 200 with code "MSG366" ("Đã xoá lượt ghi.").
+3. The audio is takes 1 and 3 back to back; the duration and the take offsets shrink by the removed take.
+4. The transcript is "Completed" with the first line and the corrected third line moved up; the name given to SPEAKER_00 stays and the voice heard only in take 2 is gone.
+5. With one take left, deleting it returns HTTP 409 "MSG367" ("Bản ghi chỉ còn một lượt ghi. Xoá cả bản ghi nếu muốn bỏ lượt này.").</v>
+      </c>
+      <c r="E79" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress in-person meeting with Secretary, Chair and Member; speech worker running.</v>
+      </c>
+      <c r="F79" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G79" s="122" t="str"/>
+      <c r="H79" s="121" t="str"/>
+      <c r="I79" s="121" t="str"/>
+      <c r="J79" s="122" t="str"/>
+      <c r="K79" s="121" t="str"/>
+      <c r="L79" s="121" t="str"/>
+      <c r="M79" s="123" t="str"/>
+      <c r="N79" s="121" t="str"/>
+      <c r="O79" s="124" t="str"/>
+      <c r="P79" s="125"/>
+      <c r="Q79" s="112"/>
+      <c r="R79" s="112"/>
+      <c r="S79" s="112"/>
+      <c r="T79" s="112"/>
+      <c r="U79" s="112"/>
+      <c r="V79" s="112"/>
+      <c r="W79" s="112"/>
+      <c r="X79" s="112"/>
+      <c r="Y79" s="112"/>
+    </row>
+    <row r="80" ht="24" customHeight="1">
+      <c r="A80" s="120" t="str">
+        <v>GET /api/recordings/{id}/download</v>
+      </c>
+      <c r="B80" s="120"/>
+      <c r="C80" s="120"/>
+      <c r="D80" s="120"/>
+      <c r="E80" s="120"/>
+      <c r="F80" s="121"/>
+      <c r="G80" s="122"/>
+      <c r="H80" s="121"/>
+      <c r="I80" s="121"/>
+      <c r="J80" s="122"/>
+      <c r="K80" s="121"/>
+      <c r="L80" s="121"/>
+      <c r="M80" s="123"/>
+      <c r="N80" s="121"/>
+      <c r="O80" s="124"/>
+      <c r="P80" s="125"/>
+      <c r="Q80" s="112"/>
+      <c r="R80" s="112"/>
+      <c r="S80" s="112"/>
+      <c r="T80" s="112"/>
+      <c r="U80" s="112"/>
+      <c r="V80" s="112"/>
+      <c r="W80" s="112"/>
+      <c r="X80" s="112"/>
+      <c r="Y80" s="112"/>
+    </row>
+    <row r="81" ht="182.0" customHeight="1">
+      <c r="A81" s="120" t="str">
+        <v>REC_API_IT42</v>
+      </c>
+      <c r="B81" s="120" t="str">
+        <v>Verify the Chair or a Secretary saves the original file and a playback link cannot be turned into one.</v>
+      </c>
+      <c r="C81" s="120" t="str">
+        <v>1. As the Member, GET the list (canDownload) and GET /api/recordings/&lt;id&gt;/download.
+2. As the Chair, GET the list and GET /api/recordings/&lt;id&gt;/download; open the returned url without signing in.
+3. As the Member, GET /api/recordings/&lt;id&gt;/playback; open its url with &amp;download=1 appended, then without it.</v>
+      </c>
+      <c r="D81" s="120" t="str">
+        <v>1. Member: canDownload is false; download returns HTTP 403 with code "MSG355" ("Chỉ Chủ tọa hoặc Thư ký được tải bản ghi và bản gỡ băng về.").
+2. Chair: canDownload is true; the url ends with &amp;download=1 and returns the original file as an attachment.
+3. The playback url with &amp;download=1 returns HTTP 404; without it, HTTP 200.
+4. The audit log records one recording.downloaded.</v>
+      </c>
+      <c r="E81" s="120" t="str">
+        <v>1. Backend is running.
+2. An Internal meeting with a stored, transcribed recording; Chair and Member on the roster.</v>
+      </c>
+      <c r="F81" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G81" s="122" t="str"/>
+      <c r="H81" s="121" t="str"/>
+      <c r="I81" s="121" t="str"/>
+      <c r="J81" s="122" t="str"/>
+      <c r="K81" s="121" t="str"/>
+      <c r="L81" s="121" t="str"/>
+      <c r="M81" s="123" t="str"/>
+      <c r="N81" s="121" t="str"/>
+      <c r="O81" s="124" t="str"/>
+      <c r="P81" s="125"/>
+      <c r="Q81" s="112"/>
+      <c r="R81" s="112"/>
+      <c r="S81" s="112"/>
+      <c r="T81" s="112"/>
+      <c r="U81" s="112"/>
+      <c r="V81" s="112"/>
+      <c r="W81" s="112"/>
+      <c r="X81" s="112"/>
+      <c r="Y81" s="112"/>
+    </row>
+    <row r="82" ht="24" customHeight="1">
+      <c r="A82" s="120" t="str">
+        <v>GET /api/recordings/{id}/transcript.txt</v>
+      </c>
+      <c r="B82" s="120"/>
+      <c r="C82" s="120"/>
+      <c r="D82" s="120"/>
+      <c r="E82" s="120"/>
+      <c r="F82" s="121"/>
+      <c r="G82" s="122"/>
+      <c r="H82" s="121"/>
+      <c r="I82" s="121"/>
+      <c r="J82" s="122"/>
+      <c r="K82" s="121"/>
+      <c r="L82" s="121"/>
+      <c r="M82" s="123"/>
+      <c r="N82" s="121"/>
+      <c r="O82" s="124"/>
+      <c r="P82" s="125"/>
+      <c r="Q82" s="112"/>
+      <c r="R82" s="112"/>
+      <c r="S82" s="112"/>
+      <c r="T82" s="112"/>
+      <c r="U82" s="112"/>
+      <c r="V82" s="112"/>
+      <c r="W82" s="112"/>
+      <c r="X82" s="112"/>
+      <c r="Y82" s="112"/>
+    </row>
+    <row r="83" ht="196.5" customHeight="1">
+      <c r="A83" s="120" t="str">
+        <v>REC_API_IT43</v>
+      </c>
+      <c r="B83" s="120" t="str">
+        <v>Verify a finished transcript is saved as text with the names the Secretary gave.</v>
+      </c>
+      <c r="C83" s="120" t="str">
+        <v>1. As the Secretary, name SPEAKER_00 as the Chair and GET the transcript (canExport).
+2. GET /api/recordings/&lt;id&gt;/transcript.txt.
+3. As the Member, GET the transcript and transcript.txt.
+4. As the Secretary, POST /api/recordings/&lt;id&gt;/transcribe, then GET transcript.txt.</v>
+      </c>
+      <c r="D83" s="120" t="str">
+        <v>1. canExport is true; the file is text/plain named ban-go-bang-…, starting with the meeting title and "Bản gỡ băng — bản ghi phien-hop.wav".
+2. Each line is "[hh:mm:ss] &lt;name&gt;: &lt;text&gt;", using the assigned name, or "Người nói N".
+3. Member: canExport is false; the file returns HTTP 403 "MSG355".
+4. Re-queueing returns HTTP 202 "MSG300"; while not finished the file returns HTTP 409 "MSG357" ("Bản gỡ băng chưa xong nên chưa tải về được.").</v>
+      </c>
+      <c r="E83" s="120" t="str">
+        <v>1. Backend is running.
+2. A recording with a completed transcript; Secretary, Chair and Member on the roster.</v>
+      </c>
+      <c r="F83" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G83" s="122" t="str"/>
+      <c r="H83" s="121" t="str"/>
+      <c r="I83" s="121" t="str"/>
+      <c r="J83" s="122" t="str"/>
+      <c r="K83" s="121" t="str"/>
+      <c r="L83" s="121" t="str"/>
+      <c r="M83" s="123" t="str"/>
+      <c r="N83" s="121" t="str"/>
+      <c r="O83" s="124" t="str"/>
+      <c r="P83" s="125"/>
+      <c r="Q83" s="112"/>
+      <c r="R83" s="112"/>
+      <c r="S83" s="112"/>
+      <c r="T83" s="112"/>
+      <c r="U83" s="112"/>
+      <c r="V83" s="112"/>
+      <c r="W83" s="112"/>
+      <c r="X83" s="112"/>
+      <c r="Y83" s="112"/>
+    </row>
+    <row r="84" ht="24" customHeight="1">
+      <c r="A84" s="120" t="str">
+        <v>GET /api/recordings/{id}/download</v>
+      </c>
+      <c r="B84" s="120"/>
+      <c r="C84" s="120"/>
+      <c r="D84" s="120"/>
+      <c r="E84" s="120"/>
+      <c r="F84" s="121"/>
+      <c r="G84" s="122"/>
+      <c r="H84" s="121"/>
+      <c r="I84" s="121"/>
+      <c r="J84" s="122"/>
+      <c r="K84" s="121"/>
+      <c r="L84" s="121"/>
+      <c r="M84" s="123"/>
+      <c r="N84" s="121"/>
+      <c r="O84" s="124"/>
+      <c r="P84" s="125"/>
+      <c r="Q84" s="112"/>
+      <c r="R84" s="112"/>
+      <c r="S84" s="112"/>
+      <c r="T84" s="112"/>
+      <c r="U84" s="112"/>
+      <c r="V84" s="112"/>
+      <c r="W84" s="112"/>
+      <c r="X84" s="112"/>
+      <c r="Y84" s="112"/>
+    </row>
+    <row r="85" ht="109.5" customHeight="1">
+      <c r="A85" s="120" t="str">
+        <v>REC_API_IT44</v>
+      </c>
+      <c r="B85" s="120" t="str">
+        <v>Verify a Secret meeting keeps its audio and words inside.</v>
+      </c>
+      <c r="C85" s="120" t="str">
+        <v>1. Mark the meeting Mật.
+2. As the Chair, GET /api/recordings/&lt;id&gt;/download, /api/recordings/&lt;id&gt;/transcript.txt and /api/meetings/&lt;id&gt;/speech-clips.txt.
+3. GET the list.</v>
+      </c>
+      <c r="D85" s="120" t="str">
+        <v>1. Each export returns HTTP 403 with code "MSG356" ("Bản ghi và bản gỡ băng của cuộc họp Mật không được tải về.").
+2. canDownload is false.</v>
+      </c>
+      <c r="E85" s="120" t="str">
+        <v>1. Backend is running.
+2. A Secret meeting with a transcribed recording; signed in as its Chair.</v>
+      </c>
+      <c r="F85" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G85" s="122" t="str"/>
+      <c r="H85" s="121" t="str"/>
+      <c r="I85" s="121" t="str"/>
+      <c r="J85" s="122" t="str"/>
+      <c r="K85" s="121" t="str"/>
+      <c r="L85" s="121" t="str"/>
+      <c r="M85" s="123" t="str"/>
+      <c r="N85" s="121" t="str"/>
+      <c r="O85" s="124" t="str"/>
+      <c r="P85" s="125"/>
+      <c r="Q85" s="112"/>
+      <c r="R85" s="112"/>
+      <c r="S85" s="112"/>
+      <c r="T85" s="112"/>
+      <c r="U85" s="112"/>
+      <c r="V85" s="112"/>
+      <c r="W85" s="112"/>
+      <c r="X85" s="112"/>
+      <c r="Y85" s="112"/>
+    </row>
+    <row r="86" ht="24" customHeight="1">
+      <c r="A86" s="120" t="str">
+        <v>GET /api/meetings/{id}/speech-clips.txt</v>
+      </c>
+      <c r="B86" s="120"/>
+      <c r="C86" s="120"/>
+      <c r="D86" s="120"/>
+      <c r="E86" s="120"/>
+      <c r="F86" s="121"/>
+      <c r="G86" s="122"/>
+      <c r="H86" s="121"/>
+      <c r="I86" s="121"/>
+      <c r="J86" s="122"/>
+      <c r="K86" s="121"/>
+      <c r="L86" s="121"/>
+      <c r="M86" s="123"/>
+      <c r="N86" s="121"/>
+      <c r="O86" s="124"/>
+      <c r="P86" s="125"/>
+      <c r="Q86" s="112"/>
+      <c r="R86" s="112"/>
+      <c r="S86" s="112"/>
+      <c r="T86" s="112"/>
+      <c r="U86" s="112"/>
+      <c r="V86" s="112"/>
+      <c r="W86" s="112"/>
+      <c r="X86" s="112"/>
+      <c r="Y86" s="112"/>
+    </row>
+    <row r="87" ht="182.0" customHeight="1">
+      <c r="A87" s="120" t="str">
+        <v>REC_API_IT45</v>
+      </c>
+      <c r="B87" s="120" t="str">
+        <v>Verify the per-microphone transcript is saved without the sentences taken out.</v>
+      </c>
+      <c r="C87" s="120" t="str">
+        <v>1. As the Member, send two sentences: "Tôi đồng ý." and "Ai tắt giúp cái điều hoà.".
+2. As the Secretary, take the second out with PUT /api/speech-clips/&lt;id&gt;/exclusion { "excluded": true, "reason": "Other" }.
+3. As the Member, GET /api/meetings/&lt;id&gt;/speech-clips.txt.
+4. As the Secretary, GET the same file.</v>
+      </c>
+      <c r="D87" s="120" t="str">
+        <v>1. Member: HTTP 403 "MSG355".
+2. The Secretary's file has the line "Bản gỡ băng — ghi theo micro từng người", contains "Tôi đồng ý." with the speaker's name and does not contain the excluded sentence.
+3. The audit log records one speech_clip.exported.</v>
+      </c>
+      <c r="E87" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress Online or Hybrid meeting (captured per microphone); Secretary and Member on the roster.</v>
+      </c>
+      <c r="F87" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G87" s="122" t="str"/>
+      <c r="H87" s="121" t="str"/>
+      <c r="I87" s="121" t="str"/>
+      <c r="J87" s="122" t="str"/>
+      <c r="K87" s="121" t="str"/>
+      <c r="L87" s="121" t="str"/>
+      <c r="M87" s="123" t="str"/>
+      <c r="N87" s="121" t="str"/>
+      <c r="O87" s="124" t="str"/>
+      <c r="P87" s="125"/>
+      <c r="Q87" s="112"/>
+      <c r="R87" s="112"/>
+      <c r="S87" s="112"/>
+      <c r="T87" s="112"/>
+      <c r="U87" s="112"/>
+      <c r="V87" s="112"/>
+      <c r="W87" s="112"/>
+      <c r="X87" s="112"/>
+      <c r="Y87" s="112"/>
+    </row>
+    <row r="88" ht="24" customHeight="1">
+      <c r="A88" s="120" t="str">
+        <v>GET /api/recordings/{id}/transcript</v>
+      </c>
+      <c r="B88" s="120"/>
+      <c r="C88" s="120"/>
+      <c r="D88" s="120"/>
+      <c r="E88" s="120"/>
+      <c r="F88" s="121"/>
+      <c r="G88" s="122"/>
+      <c r="H88" s="121"/>
+      <c r="I88" s="121"/>
+      <c r="J88" s="122"/>
+      <c r="K88" s="121"/>
+      <c r="L88" s="121"/>
+      <c r="M88" s="123"/>
+      <c r="N88" s="121"/>
+      <c r="O88" s="124"/>
+      <c r="P88" s="125"/>
+      <c r="Q88" s="112"/>
+      <c r="R88" s="112"/>
+      <c r="S88" s="112"/>
+      <c r="T88" s="112"/>
+      <c r="U88" s="112"/>
+      <c r="V88" s="112"/>
+      <c r="W88" s="112"/>
+      <c r="X88" s="112"/>
+      <c r="Y88" s="112"/>
+    </row>
+    <row r="89" ht="167.5" customHeight="1">
+      <c r="A89" s="120" t="str">
+        <v>REC_API_IT46</v>
+      </c>
+      <c r="B89" s="120" t="str">
+        <v>Verify only the Secretary gets the machine's speaker guess and a correction is audited.</v>
+      </c>
+      <c r="C89" s="120" t="str">
+        <v>1. Give SPEAKER_00 a suggested person (the Chair) with score 0.91.
+2. As the Secretary, then as the Member, GET /api/recordings/&lt;id&gt;/transcript.
+3. As the Secretary, PUT /api/transcript-segments/&lt;first segment&gt; with { "text": "Kính thưa các đồng chí, hôm nay" }.</v>
+      </c>
+      <c r="D89" s="120" t="str">
+        <v>1. The Secretary sees suggestedUserId, suggestedName and suggestionScore.
+2. The Member sees all three as null.
+3. The audit log records one transcript.segment_edited.</v>
+      </c>
+      <c r="E89" s="120" t="str">
+        <v>1. Backend is running.
+2. A recording with a completed transcript; Voice ID suggestion available.</v>
+      </c>
+      <c r="F89" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G89" s="122" t="str"/>
+      <c r="H89" s="121" t="str"/>
+      <c r="I89" s="121" t="str"/>
+      <c r="J89" s="122" t="str"/>
+      <c r="K89" s="121" t="str"/>
+      <c r="L89" s="121" t="str"/>
+      <c r="M89" s="123" t="str"/>
+      <c r="N89" s="121" t="str"/>
+      <c r="O89" s="124" t="str"/>
+      <c r="P89" s="125"/>
+      <c r="Q89" s="112"/>
+      <c r="R89" s="112"/>
+      <c r="S89" s="112"/>
+      <c r="T89" s="112"/>
+      <c r="U89" s="112"/>
+      <c r="V89" s="112"/>
+      <c r="W89" s="112"/>
+      <c r="X89" s="112"/>
+      <c r="Y89" s="112"/>
+    </row>
+    <row r="90" ht="24" customHeight="1">
+      <c r="A90" s="120" t="str">
+        <v>GET /api/speech-clips/{id}/playback</v>
+      </c>
+      <c r="B90" s="120"/>
+      <c r="C90" s="120"/>
+      <c r="D90" s="120"/>
+      <c r="E90" s="120"/>
+      <c r="F90" s="121"/>
+      <c r="G90" s="122"/>
+      <c r="H90" s="121"/>
+      <c r="I90" s="121"/>
+      <c r="J90" s="122"/>
+      <c r="K90" s="121"/>
+      <c r="L90" s="121"/>
+      <c r="M90" s="123"/>
+      <c r="N90" s="121"/>
+      <c r="O90" s="124"/>
+      <c r="P90" s="125"/>
+      <c r="Q90" s="112"/>
+      <c r="R90" s="112"/>
+      <c r="S90" s="112"/>
+      <c r="T90" s="112"/>
+      <c r="U90" s="112"/>
+      <c r="V90" s="112"/>
+      <c r="W90" s="112"/>
+      <c r="X90" s="112"/>
+      <c r="Y90" s="112"/>
+    </row>
+    <row r="91" ht="298.0" customHeight="1">
+      <c r="A91" s="120" t="str">
+        <v>REC_API_IT47</v>
+      </c>
+      <c r="B91" s="120" t="str">
+        <v>Verify everyone who reads the transcript hears a sentence through a signed link.</v>
+      </c>
+      <c r="C91" s="120" t="str">
+        <v>1. As the Member, send half a second of 16 kHz mono PCM WAV.
+2. As the Chair, GET /api/meetings/&lt;id&gt;/speech-clips and read peaks.
+3. GET /api/speech-clips/&lt;id&gt;/playback and open the url without signing in.
+4. Open the url with its signature changed, the bare /audio path, and the url with /speech-clips/ replaced by /recordings/.
+5. As an outsider, the organizer, and without signing in, GET the playback; GET playback for an unknown id.
+6. Open the url after 3 hours.</v>
+      </c>
+      <c r="D91" s="120" t="str">
+        <v>1. The line has one waveform byte per 100 ms: 0, 0, 180, 180, 180.
+2. The url starts with /api/speech-clips/&lt;id&gt;/audio?expires= and returns the same audio/wav bytes.
+3. Every altered url returns HTTP 404.
+4. Outsider, organizer and unknown id: HTTP 404; not signed in: HTTP 401.
+5. The expired url returns HTTP 404.</v>
+      </c>
+      <c r="E91" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress Online or Hybrid meeting (captured per microphone); Chair and Member on the roster; an outsider and the organizer are not.</v>
+      </c>
+      <c r="F91" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G91" s="122" t="str"/>
+      <c r="H91" s="121" t="str"/>
+      <c r="I91" s="121" t="str"/>
+      <c r="J91" s="122" t="str"/>
+      <c r="K91" s="121" t="str"/>
+      <c r="L91" s="121" t="str"/>
+      <c r="M91" s="123" t="str"/>
+      <c r="N91" s="121" t="str"/>
+      <c r="O91" s="124" t="str"/>
+      <c r="P91" s="125"/>
+      <c r="Q91" s="112"/>
+      <c r="R91" s="112"/>
+      <c r="S91" s="112"/>
+      <c r="T91" s="112"/>
+      <c r="U91" s="112"/>
+      <c r="V91" s="112"/>
+      <c r="W91" s="112"/>
+      <c r="X91" s="112"/>
+      <c r="Y91" s="112"/>
+    </row>
+    <row r="92" ht="109.5" customHeight="1">
+      <c r="A92" s="120" t="str">
+        <v>REC_API_IT48</v>
+      </c>
+      <c r="B92" s="120" t="str">
+        <v>Verify a sentence taken out of the record is heard only by the Chair and the Secretary.</v>
+      </c>
+      <c r="C92" s="120" t="str">
+        <v>1. As the Chair, take a Member's sentence out (reason Other).
+2. As the Member, GET the speech clips and the sentence's playback.
+3. As the Chair, do the same.</v>
+      </c>
+      <c r="D92" s="120" t="str">
+        <v>1. Taking it out returns HTTP 200 "MSG351".
+2. Member: hasAudio is false; playback returns HTTP 404.
+3. Chair: hasAudio is true; playback returns HTTP 200.</v>
+      </c>
+      <c r="E92" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress Online or Hybrid meeting (captured per microphone) with a stored sentence.</v>
+      </c>
+      <c r="F92" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G92" s="122" t="str"/>
+      <c r="H92" s="121" t="str"/>
+      <c r="I92" s="121" t="str"/>
+      <c r="J92" s="122" t="str"/>
+      <c r="K92" s="121" t="str"/>
+      <c r="L92" s="121" t="str"/>
+      <c r="M92" s="123" t="str"/>
+      <c r="N92" s="121" t="str"/>
+      <c r="O92" s="124" t="str"/>
+      <c r="P92" s="125"/>
+      <c r="Q92" s="112"/>
+      <c r="R92" s="112"/>
+      <c r="S92" s="112"/>
+      <c r="T92" s="112"/>
+      <c r="U92" s="112"/>
+      <c r="V92" s="112"/>
+      <c r="W92" s="112"/>
+      <c r="X92" s="112"/>
+      <c r="Y92" s="112"/>
+    </row>
+    <row r="93" ht="80.5" customHeight="1">
+      <c r="A93" s="120" t="str">
+        <v>REC_API_IT49</v>
+      </c>
+      <c r="B93" s="120" t="str">
+        <v>Verify a database outage while signing a link says so.</v>
+      </c>
+      <c r="C93" s="120" t="str">
+        <v>1. Stop PostgreSQL (or make reading sentences fail).
+2. As the Member, GET /api/speech-clips/&lt;id&gt;/playback.</v>
+      </c>
+      <c r="D93" s="120" t="str">
+        <v>1. HTTP 500 with code "MSG297" ("Không tải được danh sách bản ghi.").</v>
+      </c>
+      <c r="E93" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress Online or Hybrid meeting (captured per microphone) with a stored sentence.</v>
+      </c>
+      <c r="F93" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G93" s="122" t="str"/>
+      <c r="H93" s="121" t="str"/>
+      <c r="I93" s="121" t="str"/>
+      <c r="J93" s="122" t="str"/>
+      <c r="K93" s="121" t="str"/>
+      <c r="L93" s="121" t="str"/>
+      <c r="M93" s="123" t="str"/>
+      <c r="N93" s="121" t="str"/>
+      <c r="O93" s="124" t="str"/>
+      <c r="P93" s="125"/>
+      <c r="Q93" s="112"/>
+      <c r="R93" s="112"/>
+      <c r="S93" s="112"/>
+      <c r="T93" s="112"/>
+      <c r="U93" s="112"/>
+      <c r="V93" s="112"/>
+      <c r="W93" s="112"/>
+      <c r="X93" s="112"/>
+      <c r="Y93" s="112"/>
+    </row>
+    <row r="94" ht="24" customHeight="1">
+      <c r="A94" s="120" t="str">
+        <v>PUT /api/meetings/{id}/speech-clips/{clientId}</v>
+      </c>
+      <c r="B94" s="120"/>
+      <c r="C94" s="120"/>
+      <c r="D94" s="120"/>
+      <c r="E94" s="120"/>
+      <c r="F94" s="121"/>
+      <c r="G94" s="122"/>
+      <c r="H94" s="121"/>
+      <c r="I94" s="121"/>
+      <c r="J94" s="122"/>
+      <c r="K94" s="121"/>
+      <c r="L94" s="121"/>
+      <c r="M94" s="123"/>
+      <c r="N94" s="121"/>
+      <c r="O94" s="124"/>
+      <c r="P94" s="125"/>
+      <c r="Q94" s="112"/>
+      <c r="R94" s="112"/>
+      <c r="S94" s="112"/>
+      <c r="T94" s="112"/>
+      <c r="U94" s="112"/>
+      <c r="V94" s="112"/>
+      <c r="W94" s="112"/>
+      <c r="X94" s="112"/>
+      <c r="Y94" s="112"/>
+    </row>
+    <row r="95" ht="80.5" customHeight="1">
+      <c r="A95" s="120" t="str">
+        <v>REC_API_IT50</v>
+      </c>
+      <c r="B95" s="120" t="str">
+        <v>Verify a sentence the database could not store leaves no audio behind.</v>
+      </c>
+      <c r="C95" s="120" t="str">
+        <v>1. Make saving fail (stop PostgreSQL during the save).
+2. As the Member, send a sentence.</v>
+      </c>
+      <c r="D95" s="120" t="str">
+        <v>1. HTTP 503 with code "MSG304" ("Không lưu được thay đổi bản gỡ băng. Vui lòng thử lại.").
+2. No audio file is left in storage.</v>
+      </c>
+      <c r="E95" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress Online or Hybrid meeting (captured per microphone); speech worker running.</v>
+      </c>
+      <c r="F95" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G95" s="122" t="str"/>
+      <c r="H95" s="121" t="str"/>
+      <c r="I95" s="121" t="str"/>
+      <c r="J95" s="122" t="str"/>
+      <c r="K95" s="121" t="str"/>
+      <c r="L95" s="121" t="str"/>
+      <c r="M95" s="123" t="str"/>
+      <c r="N95" s="121" t="str"/>
+      <c r="O95" s="124" t="str"/>
+      <c r="P95" s="125"/>
+      <c r="Q95" s="112"/>
+      <c r="R95" s="112"/>
+      <c r="S95" s="112"/>
+      <c r="T95" s="112"/>
+      <c r="U95" s="112"/>
+      <c r="V95" s="112"/>
+      <c r="W95" s="112"/>
+      <c r="X95" s="112"/>
+      <c r="Y95" s="112"/>
+    </row>
+    <row r="96" ht="24" customHeight="1">
+      <c r="A96" s="120" t="str">
+        <v>DELETE /api/speech-clips/{id}</v>
+      </c>
+      <c r="B96" s="120"/>
+      <c r="C96" s="120"/>
+      <c r="D96" s="120"/>
+      <c r="E96" s="120"/>
+      <c r="F96" s="121"/>
+      <c r="G96" s="122"/>
+      <c r="H96" s="121"/>
+      <c r="I96" s="121"/>
+      <c r="J96" s="122"/>
+      <c r="K96" s="121"/>
+      <c r="L96" s="121"/>
+      <c r="M96" s="123"/>
+      <c r="N96" s="121"/>
+      <c r="O96" s="124"/>
+      <c r="P96" s="125"/>
+      <c r="Q96" s="112"/>
+      <c r="R96" s="112"/>
+      <c r="S96" s="112"/>
+      <c r="T96" s="112"/>
+      <c r="U96" s="112"/>
+      <c r="V96" s="112"/>
+      <c r="W96" s="112"/>
+      <c r="X96" s="112"/>
+      <c r="Y96" s="112"/>
+    </row>
+    <row r="97" ht="109.5" customHeight="1">
+      <c r="A97" s="120" t="str">
+        <v>REC_API_IT51</v>
+      </c>
+      <c r="B97" s="120" t="str">
+        <v>Verify deleting a sentence, or its retention running out, erases its audio.</v>
+      </c>
+      <c r="C97" s="120" t="str">
+        <v>1. As the Member, store two sentences.
+2. DELETE /api/speech-clips/&lt;first&gt;.
+3. Make the second 181 days old and run the retention sweep.</v>
+      </c>
+      <c r="D97" s="120" t="str">
+        <v>1. Deleting returns HTTP 200 "MSG322" ("Đã xoá câu nói."); its audio file is erased, the other stays.
+2. After the sweep, the expired sentence and its audio are gone.</v>
+      </c>
+      <c r="E97" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress Online or Hybrid meeting (captured per microphone); retention 180 days.</v>
+      </c>
+      <c r="F97" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G97" s="122" t="str"/>
+      <c r="H97" s="121" t="str"/>
+      <c r="I97" s="121" t="str"/>
+      <c r="J97" s="122" t="str"/>
+      <c r="K97" s="121" t="str"/>
+      <c r="L97" s="121" t="str"/>
+      <c r="M97" s="123" t="str"/>
+      <c r="N97" s="121" t="str"/>
+      <c r="O97" s="124" t="str"/>
+      <c r="P97" s="125"/>
+      <c r="Q97" s="112"/>
+      <c r="R97" s="112"/>
+      <c r="S97" s="112"/>
+      <c r="T97" s="112"/>
+      <c r="U97" s="112"/>
+      <c r="V97" s="112"/>
+      <c r="W97" s="112"/>
+      <c r="X97" s="112"/>
+      <c r="Y97" s="112"/>
+    </row>
+    <row r="98" ht="24" customHeight="1">
+      <c r="A98" s="120" t="str">
+        <v>GET /api/meetings/{id}/speech-clips</v>
+      </c>
+      <c r="B98" s="120"/>
+      <c r="C98" s="120"/>
+      <c r="D98" s="120"/>
+      <c r="E98" s="120"/>
+      <c r="F98" s="121"/>
+      <c r="G98" s="122"/>
+      <c r="H98" s="121"/>
+      <c r="I98" s="121"/>
+      <c r="J98" s="122"/>
+      <c r="K98" s="121"/>
+      <c r="L98" s="121"/>
+      <c r="M98" s="123"/>
+      <c r="N98" s="121"/>
+      <c r="O98" s="124"/>
+      <c r="P98" s="125"/>
+      <c r="Q98" s="112"/>
+      <c r="R98" s="112"/>
+      <c r="S98" s="112"/>
+      <c r="T98" s="112"/>
+      <c r="U98" s="112"/>
+      <c r="V98" s="112"/>
+      <c r="W98" s="112"/>
+      <c r="X98" s="112"/>
+      <c r="Y98" s="112"/>
+    </row>
+    <row r="99" ht="182.0" customHeight="1">
+      <c r="A99" s="120" t="str">
+        <v>REC_API_IT52</v>
+      </c>
+      <c r="B99" s="120" t="str">
+        <v>Verify a quiet copy of a neighbour's sentence is marked for everyone and kept.</v>
+      </c>
+      <c r="C99" s="120" t="str">
+        <v>1. As the Member, send a sentence that is a quieter copy (about 14 dB lower) of what the Chair said, 300 ms later on its clock; GET the list.
+2. A second later, as the Chair, send the original sentence.
+3. As the Member, GET the list with ?since=&lt;readAt of the first read&gt;, then the whole list.</v>
+      </c>
+      <c r="D99" s="120" t="str">
+        <v>1. Before the Chair's sentence arrives the Member's line has leak null.
+2. The ?since read returns both lines: the Member's line is marked leak with the Chair's clipId, speakerName and whole true; the Chair's line has leak null.
+3. Both lines stay in the list: the copy is marked, not hidden.</v>
+      </c>
+      <c r="E99" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress Online or Hybrid meeting (captured per microphone); Chair and Member on the roster; speech worker running.</v>
+      </c>
+      <c r="F99" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G99" s="122" t="str"/>
+      <c r="H99" s="121" t="str"/>
+      <c r="I99" s="121" t="str"/>
+      <c r="J99" s="122" t="str"/>
+      <c r="K99" s="121" t="str"/>
+      <c r="L99" s="121" t="str"/>
+      <c r="M99" s="123" t="str"/>
+      <c r="N99" s="121" t="str"/>
+      <c r="O99" s="124" t="str"/>
+      <c r="P99" s="125"/>
+      <c r="Q99" s="112"/>
+      <c r="R99" s="112"/>
+      <c r="S99" s="112"/>
+      <c r="T99" s="112"/>
+      <c r="U99" s="112"/>
+      <c r="V99" s="112"/>
+      <c r="W99" s="112"/>
+      <c r="X99" s="112"/>
+      <c r="Y99" s="112"/>
+    </row>
+    <row r="100" ht="24" customHeight="1">
+      <c r="A100" s="120" t="str">
+        <v>PUT /api/speech-clips/{id}/exclusion</v>
+      </c>
+      <c r="B100" s="120"/>
+      <c r="C100" s="120"/>
+      <c r="D100" s="120"/>
+      <c r="E100" s="120"/>
+      <c r="F100" s="121"/>
+      <c r="G100" s="122"/>
+      <c r="H100" s="121"/>
+      <c r="I100" s="121"/>
+      <c r="J100" s="122"/>
+      <c r="K100" s="121"/>
+      <c r="L100" s="121"/>
+      <c r="M100" s="123"/>
+      <c r="N100" s="121"/>
+      <c r="O100" s="124"/>
+      <c r="P100" s="125"/>
+      <c r="Q100" s="112"/>
+      <c r="R100" s="112"/>
+      <c r="S100" s="112"/>
+      <c r="T100" s="112"/>
+      <c r="U100" s="112"/>
+      <c r="V100" s="112"/>
+      <c r="W100" s="112"/>
+      <c r="X100" s="112"/>
+      <c r="Y100" s="112"/>
+    </row>
+    <row r="101" ht="254.5" customHeight="1">
+      <c r="A101" s="120" t="str">
+        <v>REC_API_IT53</v>
+      </c>
+      <c r="B101" s="120" t="str">
+        <v>Verify the Chair or a Secretary takes a sentence out of the record and puts it back.</v>
+      </c>
+      <c r="C101" s="120" t="str">
+        <v>1. As the Member, GET the list (canExclude) and PUT /api/speech-clips/&lt;id&gt;/exclusion { "excluded": true, "reason": "Leak" }.
+2. As the Chair, PUT with reason "Rò rỉ", then with "Leak" twice.
+3. As the Chair and as the Member, GET the list.
+4. As the Secretary, PUT { "excluded": false }.
+5. PUT for an unknown id.</v>
+      </c>
+      <c r="D101" s="120" t="str">
+        <v>1. Member: canExclude is false; HTTP 403 "MSG353" ("Chỉ Chủ tọa hoặc Thư ký được loại câu khỏi bản ghi.").
+2. Wrong reason: HTTP 400 "MSG354" ("Lý do loại câu không hợp lệ."). Valid: HTTP 200 "MSG351" ("Đã loại câu khỏi bản ghi."); the second tap changes nothing.
+3. The Chair sees the words, the reason and who took it out; the Member sees an excluded line with empty text and no name.
+4. Putting back returns HTTP 200 "MSG352" ("Đã đưa câu trở lại bản ghi."); the audit log has speech_clip.excluded then speech_clip.restored.
+5. Unknown id: HTTP 404.</v>
+      </c>
+      <c r="E101" s="120" t="str">
+        <v>1. Backend is running.
+2. An InProgress Online or Hybrid meeting (captured per microphone) with a stored sentence; Chair, Secretary and Member on the roster.</v>
+      </c>
+      <c r="F101" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G101" s="122" t="str"/>
+      <c r="H101" s="121" t="str"/>
+      <c r="I101" s="121" t="str"/>
+      <c r="J101" s="122" t="str"/>
+      <c r="K101" s="121" t="str"/>
+      <c r="L101" s="121" t="str"/>
+      <c r="M101" s="123" t="str"/>
+      <c r="N101" s="121" t="str"/>
+      <c r="O101" s="124" t="str"/>
+      <c r="P101" s="125"/>
+      <c r="Q101" s="112"/>
+      <c r="R101" s="112"/>
+      <c r="S101" s="112"/>
+      <c r="T101" s="112"/>
+      <c r="U101" s="112"/>
+      <c r="V101" s="112"/>
+      <c r="W101" s="112"/>
+      <c r="X101" s="112"/>
+      <c r="Y101" s="112"/>
+    </row>
+    <row r="102" ht="24" customHeight="1">
+      <c r="A102" s="120" t="str">
+        <v>PUT /api/meetings/{id}/speech-clips/{clientId}</v>
+      </c>
+      <c r="B102" s="120"/>
+      <c r="C102" s="120"/>
+      <c r="D102" s="120"/>
+      <c r="E102" s="120"/>
+      <c r="F102" s="121"/>
+      <c r="G102" s="122"/>
+      <c r="H102" s="121"/>
+      <c r="I102" s="121"/>
+      <c r="J102" s="122"/>
+      <c r="K102" s="121"/>
+      <c r="L102" s="121"/>
+      <c r="M102" s="123"/>
+      <c r="N102" s="121"/>
+      <c r="O102" s="124"/>
+      <c r="P102" s="125"/>
+      <c r="Q102" s="112"/>
+      <c r="R102" s="112"/>
+      <c r="S102" s="112"/>
+      <c r="T102" s="112"/>
+      <c r="U102" s="112"/>
+      <c r="V102" s="112"/>
+      <c r="W102" s="112"/>
+      <c r="X102" s="112"/>
+      <c r="Y102" s="112"/>
+    </row>
+    <row r="103" ht="167.5" customHeight="1">
+      <c r="A103" s="120" t="str">
+        <v>REC_API_IT54</v>
+      </c>
+      <c r="B103" s="120" t="str">
+        <v>Verify a sentence kept on the device still arrives up to a week after the meeting.</v>
+      </c>
+      <c r="C103" s="120" t="str">
+        <v>1. End the meeting one day ago.
+2. As the Member, GET the list (canCapture), then send a sentence said 5 minutes before the end.
+3. Send a sentence whose startedAt is after the meeting ended.
+4. Move the end beyond the 7-day window and send again.</v>
+      </c>
+      <c r="D103" s="120" t="str">
+        <v>1. canCapture is false, yet the late sentence returns HTTP 200 "MSG318" with its own startedAt.
+2. A sentence dated after the end is saved as ending when the meeting ended.
+3. Past 7 days: HTTP 409 "MSG320".</v>
+      </c>
+      <c r="E103" s="120" t="str">
+        <v>1. Backend is running.
+2. An Ended Online meeting with the Member on its roster; speech worker running.</v>
+      </c>
+      <c r="F103" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G103" s="122" t="str"/>
+      <c r="H103" s="121" t="str"/>
+      <c r="I103" s="121" t="str"/>
+      <c r="J103" s="122" t="str"/>
+      <c r="K103" s="121" t="str"/>
+      <c r="L103" s="121" t="str"/>
+      <c r="M103" s="123" t="str"/>
+      <c r="N103" s="121" t="str"/>
+      <c r="O103" s="124" t="str"/>
+      <c r="P103" s="125"/>
+      <c r="Q103" s="112"/>
+      <c r="R103" s="112"/>
+      <c r="S103" s="112"/>
+      <c r="T103" s="112"/>
+      <c r="U103" s="112"/>
+      <c r="V103" s="112"/>
+      <c r="W103" s="112"/>
+      <c r="X103" s="112"/>
+      <c r="Y103" s="112"/>
+    </row>
+    <row r="104" ht="24" customHeight="1">
+      <c r="A104" s="120" t="str">
+        <v>GET /api/me/voice/samples/{id}/audio</v>
+      </c>
+      <c r="B104" s="120"/>
+      <c r="C104" s="120"/>
+      <c r="D104" s="120"/>
+      <c r="E104" s="120"/>
+      <c r="F104" s="121"/>
+      <c r="G104" s="122"/>
+      <c r="H104" s="121"/>
+      <c r="I104" s="121"/>
+      <c r="J104" s="122"/>
+      <c r="K104" s="121"/>
+      <c r="L104" s="121"/>
+      <c r="M104" s="123"/>
+      <c r="N104" s="121"/>
+      <c r="O104" s="124"/>
+      <c r="P104" s="125"/>
+      <c r="Q104" s="112"/>
+      <c r="R104" s="112"/>
+      <c r="S104" s="112"/>
+      <c r="T104" s="112"/>
+      <c r="U104" s="112"/>
+      <c r="V104" s="112"/>
+      <c r="W104" s="112"/>
+      <c r="X104" s="112"/>
+      <c r="Y104" s="112"/>
+    </row>
+    <row r="105" ht="196.5" customHeight="1">
+      <c r="A105" s="120" t="str">
+        <v>REC_API_IT55</v>
+      </c>
+      <c r="B105" s="120" t="str">
+        <v>Verify a sample recording is kept only under the newer notice and only its owner hears it.</v>
+      </c>
+      <c r="C105" s="120" t="str">
+        <v>1. With consent to notice 1.0, POST /api/me/voice/samples and GET its /audio.
+2. POST /api/me/voice/consent with the current noticeVersion.
+3. POST another sample and GET /api/me/voice/samples/&lt;id&gt;/audio.
+4. As another user, then without signing in, GET the same /audio.</v>
+      </c>
+      <c r="D105" s="120" t="str">
+        <v>1. The old sample returns HTTP 201 "MSG307" with playable false; its audio returns HTTP 404.
+2. Renewing returns HTTP 200 "MSG305" with the current noticeVersion; the existing sample stays and the same consent row is renewed (audited).
+3. The new sample is playable; its audio returns HTTP 200 audio/webm with Cache-Control no-store; the stored copy is encrypted.
+4. Another user: HTTP 404. Not signed in: HTTP 401.</v>
+      </c>
+      <c r="E105" s="120" t="str">
+        <v>1. Backend is running.
+2. Signed in as thanhvien@trustcabinet.local, who agreed to the earlier notice 1.0; speech worker running.</v>
+      </c>
+      <c r="F105" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G105" s="122" t="str"/>
+      <c r="H105" s="121" t="str"/>
+      <c r="I105" s="121" t="str"/>
+      <c r="J105" s="122" t="str"/>
+      <c r="K105" s="121" t="str"/>
+      <c r="L105" s="121" t="str"/>
+      <c r="M105" s="123" t="str"/>
+      <c r="N105" s="121" t="str"/>
+      <c r="O105" s="124" t="str"/>
+      <c r="P105" s="125"/>
+      <c r="Q105" s="112"/>
+      <c r="R105" s="112"/>
+      <c r="S105" s="112"/>
+      <c r="T105" s="112"/>
+      <c r="U105" s="112"/>
+      <c r="V105" s="112"/>
+      <c r="W105" s="112"/>
+      <c r="X105" s="112"/>
+      <c r="Y105" s="112"/>
+    </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="43">
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B4:E4"/>
@@ -17497,6 +19137,25 @@
     <mergeCell ref="A57:O57"/>
     <mergeCell ref="A59:O59"/>
     <mergeCell ref="A61:O61"/>
+    <mergeCell ref="A63:O63"/>
+    <mergeCell ref="A65:O65"/>
+    <mergeCell ref="A68:O68"/>
+    <mergeCell ref="A70:O70"/>
+    <mergeCell ref="A72:O72"/>
+    <mergeCell ref="A75:O75"/>
+    <mergeCell ref="A78:O78"/>
+    <mergeCell ref="A80:O80"/>
+    <mergeCell ref="A82:O82"/>
+    <mergeCell ref="A84:O84"/>
+    <mergeCell ref="A86:O86"/>
+    <mergeCell ref="A88:O88"/>
+    <mergeCell ref="A90:O90"/>
+    <mergeCell ref="A94:O94"/>
+    <mergeCell ref="A96:O96"/>
+    <mergeCell ref="A98:O98"/>
+    <mergeCell ref="A100:O100"/>
+    <mergeCell ref="A102:O102"/>
+    <mergeCell ref="A104:O104"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.9840277777777777" footer="0.0" header="0.0" left="0.7479166666666667" right="0.25" top="0.75"/>
@@ -19896,7 +21555,7 @@
         <v>Agenda</v>
       </c>
       <c r="E10" s="65" t="str">
-        <v>55 definitions / scenarios</v>
+        <v>57 definitions / scenarios</v>
       </c>
       <c r="F10" s="66" t="str">
         <v>See the Pre-conditions of each case.</v>
@@ -20276,7 +21935,7 @@
         <v>Recordings</v>
       </c>
       <c r="E20" s="65" t="str">
-        <v>31 definitions / scenarios</v>
+        <v>55 definitions / scenarios</v>
       </c>
       <c r="F20" s="66" t="str">
         <v>See the Pre-conditions of each case.</v>
@@ -20525,7 +22184,7 @@
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="83" t="str">
-        <v>2026-10-29</v>
+        <v>2026-10-30</v>
       </c>
       <c r="H5" s="6"/>
       <c r="I5" s="10"/>
@@ -20768,7 +22427,7 @@
       </c>
       <c r="F12" s="94" t="n">
         <f>'Agenda'!D6</f>
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G12" s="94" t="n">
         <f>'Agenda'!E6</f>
@@ -20776,7 +22435,7 @@
       </c>
       <c r="H12" s="95" t="n">
         <f>'Agenda'!B4</f>
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I12" s="49"/>
       <c r="J12" s="10"/>
@@ -21238,7 +22897,7 @@
       </c>
       <c r="F22" s="94" t="n">
         <f>'Recordings'!D6</f>
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="G22" s="94" t="n">
         <f>'Recordings'!E6</f>
@@ -21246,7 +22905,7 @@
       </c>
       <c r="H22" s="95" t="n">
         <f>'Recordings'!B4</f>
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="I22" s="49"/>
       <c r="J22" s="10"/>
@@ -21330,7 +22989,7 @@
       </c>
       <c r="F24" s="100" t="n">
         <f>SUM(F11:F23)</f>
-        <v>453</v>
+        <v>479</v>
       </c>
       <c r="G24" s="100" t="n">
         <f>SUM(G11:G23)</f>
@@ -21338,7 +22997,7 @@
       </c>
       <c r="H24" s="101" t="n">
         <f>SUM(H11:H23)</f>
-        <v>453</v>
+        <v>479</v>
       </c>
       <c r="I24" s="10"/>
       <c r="Q24" s="10"/>
@@ -24667,7 +26326,7 @@
         <v>Number of TCs</v>
       </c>
       <c r="B4" s="110" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -24739,19 +26398,19 @@
         <v>Round 1</v>
       </c>
       <c r="B6" s="114" t="n">
-        <f>COUNTIF(F12:F102,"Passed")</f>
+        <f>COUNTIF(F12:F106,"Passed")</f>
         <v>0</v>
       </c>
       <c r="C6" s="114" t="n">
-        <f>COUNTIF(F12:F102,"Failed")</f>
+        <f>COUNTIF(F12:F106,"Failed")</f>
         <v>0</v>
       </c>
       <c r="D6" s="114" t="n">
         <f>B4-B6-C6-E6</f>
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E6" s="114" t="n">
-        <f>COUNTIF(F12:F102,"Skipped")</f>
+        <f>COUNTIF(F12:F106,"Skipped")</f>
         <v>0</v>
       </c>
       <c r="F6" s="107"/>
@@ -24780,19 +26439,19 @@
         <v>Round 2</v>
       </c>
       <c r="B7" s="114" t="n">
-        <f>COUNTIF(I12:I102,"Passed")</f>
+        <f>COUNTIF(I12:I106,"Passed")</f>
         <v>0</v>
       </c>
       <c r="C7" s="114" t="n">
-        <f>COUNTIF(I12:I102,"Failed")</f>
+        <f>COUNTIF(I12:I106,"Failed")</f>
         <v>0</v>
       </c>
       <c r="D7" s="114" t="n">
         <f>B4-B7-C7-E7</f>
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E7" s="114" t="n">
-        <f>COUNTIF(I12:I102,"Skipped")</f>
+        <f>COUNTIF(I12:I106,"Skipped")</f>
         <v>0</v>
       </c>
       <c r="F7" s="107"/>
@@ -24821,19 +26480,19 @@
         <v>Round 3</v>
       </c>
       <c r="B8" s="114" t="n">
-        <f>COUNTIF(L12:L102,"Passed")</f>
+        <f>COUNTIF(L12:L106,"Passed")</f>
         <v>0</v>
       </c>
       <c r="C8" s="114" t="n">
-        <f>COUNTIF(L12:L102,"Failed")</f>
+        <f>COUNTIF(L12:L106,"Failed")</f>
         <v>0</v>
       </c>
       <c r="D8" s="114" t="n">
         <f>B4-B8-C8-E8</f>
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E8" s="114" t="n">
-        <f>COUNTIF(L12:L102,"Skipped")</f>
+        <f>COUNTIF(L12:L106,"Skipped")</f>
         <v>0</v>
       </c>
       <c r="F8" s="107"/>
@@ -28345,8 +30004,155 @@
       <c r="X102" s="112"/>
       <c r="Y102" s="112"/>
     </row>
+    <row r="103" ht="24" customHeight="1">
+      <c r="A103" s="120" t="str">
+        <v>PUT /api/meetings/{id}/agenda/{itemId}</v>
+      </c>
+      <c r="B103" s="120"/>
+      <c r="C103" s="120"/>
+      <c r="D103" s="120"/>
+      <c r="E103" s="120"/>
+      <c r="F103" s="121"/>
+      <c r="G103" s="122"/>
+      <c r="H103" s="121"/>
+      <c r="I103" s="121"/>
+      <c r="J103" s="122"/>
+      <c r="K103" s="121"/>
+      <c r="L103" s="121"/>
+      <c r="M103" s="123"/>
+      <c r="N103" s="121"/>
+      <c r="O103" s="124"/>
+      <c r="P103" s="125"/>
+      <c r="Q103" s="112"/>
+      <c r="R103" s="112"/>
+      <c r="S103" s="112"/>
+      <c r="T103" s="112"/>
+      <c r="U103" s="112"/>
+      <c r="V103" s="112"/>
+      <c r="W103" s="112"/>
+      <c r="X103" s="112"/>
+      <c r="Y103" s="112"/>
+    </row>
+    <row r="104" ht="211.0" customHeight="1">
+      <c r="A104" s="120" t="str">
+        <v>AGD_API_IT56</v>
+      </c>
+      <c r="B104" s="120" t="str">
+        <v>Verify an update without documentIds keeps the links and an empty list clears them.</v>
+      </c>
+      <c r="C104" s="120" t="str">
+        <v>1. As the Secretary, PUT /api/meetings/&lt;id&gt;/agenda/&lt;item&gt; linking one meeting document.
+2. PUT with { "title": "Tiêu đề", "description": "Dòng 1\nDòng 2" } (no change).
+3. PUT { "title": "Đổi tên" }, then { "title": "Đổi tên", "documentIds": null }.
+4. PUT with "documentIds": [].
+5. POST /api/meetings/&lt;id&gt;/agenda { "title": "Mới" } and GET the agenda.</v>
+      </c>
+      <c r="D104" s="120" t="str">
+        <v>1. Every PUT returns HTTP 200 with code "MSG61" ("Cập nhật mục nghị sự thành công."); the unchanged update sends no realtime event.
+2. Omitting documentIds, or sending null, keeps the document linked to the item.
+3. An empty list unlinks it; the document itself stays in the meeting.
+4. The new item returns HTTP 201 "MSG60" and has no documents.</v>
+      </c>
+      <c r="E104" s="120" t="str">
+        <v>1. Backend is running.
+2. A meeting with an agenda item and one meeting document; signed in as its Secretary.</v>
+      </c>
+      <c r="F104" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G104" s="122" t="str"/>
+      <c r="H104" s="121" t="str"/>
+      <c r="I104" s="121" t="str"/>
+      <c r="J104" s="122" t="str"/>
+      <c r="K104" s="121" t="str"/>
+      <c r="L104" s="121" t="str"/>
+      <c r="M104" s="123" t="str"/>
+      <c r="N104" s="121" t="str"/>
+      <c r="O104" s="124" t="str"/>
+      <c r="P104" s="125"/>
+      <c r="Q104" s="112"/>
+      <c r="R104" s="112"/>
+      <c r="S104" s="112"/>
+      <c r="T104" s="112"/>
+      <c r="U104" s="112"/>
+      <c r="V104" s="112"/>
+      <c r="W104" s="112"/>
+      <c r="X104" s="112"/>
+      <c r="Y104" s="112"/>
+    </row>
+    <row r="105" ht="24" customHeight="1">
+      <c r="A105" s="120" t="str">
+        <v>GET /api/meetings/{id}/agenda</v>
+      </c>
+      <c r="B105" s="120"/>
+      <c r="C105" s="120"/>
+      <c r="D105" s="120"/>
+      <c r="E105" s="120"/>
+      <c r="F105" s="121"/>
+      <c r="G105" s="122"/>
+      <c r="H105" s="121"/>
+      <c r="I105" s="121"/>
+      <c r="J105" s="122"/>
+      <c r="K105" s="121"/>
+      <c r="L105" s="121"/>
+      <c r="M105" s="123"/>
+      <c r="N105" s="121"/>
+      <c r="O105" s="124"/>
+      <c r="P105" s="125"/>
+      <c r="Q105" s="112"/>
+      <c r="R105" s="112"/>
+      <c r="S105" s="112"/>
+      <c r="T105" s="112"/>
+      <c r="U105" s="112"/>
+      <c r="V105" s="112"/>
+      <c r="W105" s="112"/>
+      <c r="X105" s="112"/>
+      <c r="Y105" s="112"/>
+    </row>
+    <row r="106" ht="124.0" customHeight="1">
+      <c r="A106" s="120" t="str">
+        <v>AGD_API_IT57</v>
+      </c>
+      <c r="B106" s="120" t="str">
+        <v>Verify canLinkDocuments follows the document rules, not agenda planning (Published, InProgress, Ended).</v>
+      </c>
+      <c r="C106" s="120" t="str">
+        <v>1. For a Published meeting, GET /api/meetings/&lt;id&gt;/agenda as the Chair, the Secretary, a Member and the organizer; read items[0].actions.canLinkDocuments.
+2. Repeat for an InProgress and an Ended meeting.</v>
+      </c>
+      <c r="D106" s="120" t="str">
+        <v>1. Published and InProgress: true for the Chair and the Secretary; false for the Member and the organizer.
+2. Ended: false for everyone.</v>
+      </c>
+      <c r="E106" s="120" t="str">
+        <v>1. Backend is running.
+2. Meetings in each status with one agenda item; Chair, Secretary and Member on the roster; the organizer is not.</v>
+      </c>
+      <c r="F106" s="121" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G106" s="122" t="str"/>
+      <c r="H106" s="121" t="str"/>
+      <c r="I106" s="121" t="str"/>
+      <c r="J106" s="122" t="str"/>
+      <c r="K106" s="121" t="str"/>
+      <c r="L106" s="121" t="str"/>
+      <c r="M106" s="123" t="str"/>
+      <c r="N106" s="121" t="str"/>
+      <c r="O106" s="124" t="str"/>
+      <c r="P106" s="125"/>
+      <c r="Q106" s="112"/>
+      <c r="R106" s="112"/>
+      <c r="S106" s="112"/>
+      <c r="T106" s="112"/>
+      <c r="U106" s="112"/>
+      <c r="V106" s="112"/>
+      <c r="W106" s="112"/>
+      <c r="X106" s="112"/>
+      <c r="Y106" s="112"/>
+    </row>
   </sheetData>
-  <mergeCells count="40">
+  <mergeCells count="42">
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B4:E4"/>
@@ -28387,6 +30193,8 @@
     <mergeCell ref="A94:O94"/>
     <mergeCell ref="A99:O99"/>
     <mergeCell ref="A101:O101"/>
+    <mergeCell ref="A103:O103"/>
+    <mergeCell ref="A105:O105"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.9840277777777777" footer="0.0" header="0.0" left="0.7479166666666667" right="0.25" top="0.75"/>

</xml_diff>